<commit_message>
Amplía el archivo de ejemplo con problemas a las reglas nuevas
Importar-correctos.xlsx ya cumplía y se queda igual: cinco filas nuevas,
sin incidencias y con Continuar.

Importar-incompletos.xlsx solo ejercitaba siete códigos y ninguno de los
que añadieron las últimas reglas. Pasa a diecinueve filas que recorren el
catálogo entero: una incidencia clara por fila para VAL-EST-004/005/006,
VAL-MAE-001/002, VAL-GS1-002/003/004/005 y VAL-EMP-001/002, más los pares
que necesitan las reglas de unicidad VAL-UNI-001/003/004.

Cierra con dos filas No GS1 de mismo código y proveedores distintos, el
caso CF-51775-29: no son incidencia, se cuentan como nuevas y no se
listan, de modo que el archivo también demuestra que la tabla solo
enseña las filas con incidencia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJrqS6Z27X2jyr3npi3vA3
</commit_message>
<xml_diff>
--- a/ejemplos/Importar-incompletos.xlsx
+++ b/ejemplos/Importar-incompletos.xlsx
@@ -426,13 +426,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -489,12 +489,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GS1</t>
+          <t>No GS1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>7501234567893</t>
+          <t>PROP-A-001</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -522,17 +522,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gates de México</t>
+          <t>Mann-Filter México</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GS1</t>
+          <t>No GS1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>7501234567893</t>
+          <t>PROP-A-002</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -565,12 +565,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GS1</t>
+          <t>No GS1</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>7501234567893</t>
+          <t>PROP-A-003</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -608,12 +608,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>7501234567899</t>
+          <t>7501234567890</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Producto</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -621,10 +621,8 @@
           <t>Unidad</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
+      <c r="G5" t="n">
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -648,22 +646,556 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>75012345678</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1256613</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Timken Rodamientos</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GS1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>(01)07501234567893</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Surtido</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>doce</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Suspendido</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1001000</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Brembo Frenos</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GS1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>007501234567890123</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1023711</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sachs Embragues</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>PROP-A-007</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1054701</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TRW Frenos</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>PROP-A-008</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Presentación</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1175731</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Valeo Service</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>PPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPP</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1256613</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Gates de México</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D12" s="2">
+        <f>A1</f>
+        <v/>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1001000</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Moog Suspensiones</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GS1</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>7501555444330</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1001000</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Moog Suspensiones</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GS1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>7501555444330</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1023711</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SKF Rodamientos</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GS1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>7501999888776</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1054701</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Hella Iluminación</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>GS1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>7501999888776</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Presentación</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>48</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1175731</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Aisin Autopartes</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>PROP-B-100</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1256613</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Aisin Autopartes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>PROP-B-100</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Presentación</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Inner</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1001000</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dana Transmisiones</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>PROP-C-200</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1023711</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Delphi Technologies</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>No GS1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>PROP-C-200</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Presentación</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>96</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
     </row>

</xml_diff>